<commit_message>
Add RC stair forms, landings and explicit reinforcement connections
</commit_message>
<xml_diff>
--- a/examples/extensions/thai_bim/examples/slab-reinforcement-BBS.xlsx
+++ b/examples/extensions/thai_bim/examples/slab-reinforcement-BBS.xlsx
@@ -164,12 +164,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-4E26E3FCA12B</t>
+          <t xml:space="preserve">B-4068504360E9</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -181,26 +181,26 @@
         <v>12.0</v>
       </c>
       <c r="E2" s="2">
-        <v>11.0</v>
+        <v>7.0</v>
       </c>
       <c r="F2" s="2">
-        <v>0.5</v>
+        <v>2.9380000001999997</v>
       </c>
       <c r="G2" s="2">
-        <v>5.5</v>
+        <v>20.5660000014</v>
       </c>
       <c r="H2" s="2">
         <v>0.8878140839044755</v>
       </c>
       <c r="I2" s="2">
-        <v>4.882977461474615</v>
+        <v>18.258784450822382</v>
       </c>
       <c r="J2" s="2">
         <v>6.0</v>
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">500.000</t>
+          <t xml:space="preserve">2938.000</t>
         </is>
       </c>
       <c r="L2" s="0" t="inlineStr">
@@ -213,7 +213,7 @@
       </c>
       <c r="N2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="O2" s="0" t="inlineStr">
@@ -238,12 +238,12 @@
       </c>
       <c r="S2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">End dowel Start</t>
+          <t xml:space="preserve">Main Bottom</t>
         </is>
       </c>
       <c r="U2" s="0" t="inlineStr">
@@ -255,12 +255,12 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-A359E7AF0105</t>
+          <t xml:space="preserve">B-54ED5FEFBD3F</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -269,29 +269,29 @@
         </is>
       </c>
       <c r="D3" s="2">
-        <v>3.0</v>
+        <v>12.0</v>
       </c>
       <c r="E3" s="2">
-        <v>21.0</v>
+        <v>14.0</v>
       </c>
       <c r="F3" s="2">
-        <v>1.9470000002</v>
+        <v>1.9380000002</v>
       </c>
       <c r="G3" s="2">
-        <v>40.887000004200004</v>
+        <v>27.132000002799998</v>
       </c>
       <c r="H3" s="2">
-        <v>0.05548838024402972</v>
+        <v>0.8878140839044755</v>
       </c>
       <c r="I3" s="2">
-        <v>2.2687534032706944</v>
+        <v>24.08817172698211</v>
       </c>
       <c r="J3" s="2">
-        <v>1.5</v>
+        <v>6.0</v>
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1947.000</t>
+          <t xml:space="preserve">1938.000</t>
         </is>
       </c>
       <c r="L3" s="0" t="inlineStr">
@@ -304,7 +304,7 @@
       </c>
       <c r="N3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="O3" s="0" t="inlineStr">
@@ -329,29 +329,29 @@
       </c>
       <c r="S3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wire mesh B</t>
+          <t xml:space="preserve">Main Bottom</t>
         </is>
       </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-D6B42F9271BC</t>
+          <t xml:space="preserve">B-74C88A2DAA56</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -360,29 +360,29 @@
         </is>
       </c>
       <c r="D4" s="2">
-        <v>12.0</v>
+        <v>6.0</v>
       </c>
       <c r="E4" s="2">
-        <v>11.0</v>
+        <v>1.0</v>
       </c>
       <c r="F4" s="2">
-        <v>0.5</v>
+        <v>0.9456013470417681</v>
       </c>
       <c r="G4" s="2">
-        <v>5.5</v>
+        <v>0.9456013470417681</v>
       </c>
       <c r="H4" s="2">
-        <v>0.8878140839044755</v>
+        <v>0.22195352097611887</v>
       </c>
       <c r="I4" s="2">
-        <v>4.882977461474615</v>
+        <v>0.20987954841568132</v>
       </c>
       <c r="J4" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">500.000</t>
+          <t xml:space="preserve">945.601</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
@@ -395,7 +395,7 @@
       </c>
       <c r="N4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="O4" s="0" t="inlineStr">
@@ -420,12 +420,12 @@
       </c>
       <c r="S4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">End dowel End</t>
+          <t xml:space="preserve">Distribution Bottom</t>
         </is>
       </c>
       <c r="U4" s="0" t="inlineStr">
@@ -437,12 +437,12 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-DCB1303E84A9</t>
+          <t xml:space="preserve">B-C737C991D2B6</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -451,29 +451,29 @@
         </is>
       </c>
       <c r="D5" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.9440000002</v>
+      </c>
+      <c r="G5" s="2">
+        <v>4.720000001</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0.22195352097611887</v>
+      </c>
+      <c r="I5" s="2">
+        <v>1.0476206192292348</v>
+      </c>
+      <c r="J5" s="2">
         <v>3.0</v>
       </c>
-      <c r="E5" s="2">
-        <v>14.0</v>
-      </c>
-      <c r="F5" s="2">
-        <v>2.9470000002</v>
-      </c>
-      <c r="G5" s="2">
-        <v>41.2580000028</v>
-      </c>
-      <c r="H5" s="2">
-        <v>0.05548838024402972</v>
-      </c>
-      <c r="I5" s="2">
-        <v>2.289339592263546</v>
-      </c>
-      <c r="J5" s="2">
-        <v>1.5</v>
-      </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2947.000</t>
+          <t xml:space="preserve">944.000</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="N5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="O5" s="0" t="inlineStr">
@@ -511,17 +511,17 @@
       </c>
       <c r="S5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wire mesh A</t>
+          <t xml:space="preserve">Distribution Bottom</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-4068504360E9</t>
+          <t xml:space="preserve">B-EC740FDBD18C</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -542,29 +542,29 @@
         </is>
       </c>
       <c r="D6" s="2">
-        <v>12.0</v>
+        <v>6.0</v>
       </c>
       <c r="E6" s="2">
-        <v>7.0</v>
+        <v>10.0</v>
       </c>
       <c r="F6" s="2">
-        <v>2.9380000001999997</v>
+        <v>2.9440000002</v>
       </c>
       <c r="G6" s="2">
-        <v>20.5660000014</v>
+        <v>29.440000001999998</v>
       </c>
       <c r="H6" s="2">
-        <v>0.8878140839044755</v>
+        <v>0.22195352097611887</v>
       </c>
       <c r="I6" s="2">
-        <v>18.258784450822382</v>
+        <v>6.534311657980847</v>
       </c>
       <c r="J6" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2938.000</t>
+          <t xml:space="preserve">2944.000</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="N6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="O6" s="0" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="T6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main Bottom</t>
+          <t xml:space="preserve">Distribution Bottom</t>
         </is>
       </c>
       <c r="U6" s="0" t="inlineStr">
@@ -619,12 +619,12 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-54ED5FEFBD3F</t>
+          <t xml:space="preserve">B-4E26E3FCA12B</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -636,26 +636,26 @@
         <v>12.0</v>
       </c>
       <c r="E7" s="2">
-        <v>14.0</v>
+        <v>11.0</v>
       </c>
       <c r="F7" s="2">
-        <v>1.9380000002</v>
+        <v>0.5</v>
       </c>
       <c r="G7" s="2">
-        <v>27.132000002799998</v>
+        <v>5.5</v>
       </c>
       <c r="H7" s="2">
         <v>0.8878140839044755</v>
       </c>
       <c r="I7" s="2">
-        <v>24.08817172698211</v>
+        <v>4.882977461474615</v>
       </c>
       <c r="J7" s="2">
         <v>6.0</v>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1938.000</t>
+          <t xml:space="preserve">500.000</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="N7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="O7" s="0" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="S7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main Bottom</t>
+          <t xml:space="preserve">End dowel Start</t>
         </is>
       </c>
       <c r="U7" s="0" t="inlineStr">
@@ -710,12 +710,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-74C88A2DAA56</t>
+          <t xml:space="preserve">B-A359E7AF0105</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -724,29 +724,29 @@
         </is>
       </c>
       <c r="D8" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="E8" s="2">
-        <v>1.0</v>
+        <v>21.0</v>
       </c>
       <c r="F8" s="2">
-        <v>0.9456013470417681</v>
+        <v>1.9470000002</v>
       </c>
       <c r="G8" s="2">
-        <v>0.9456013470417681</v>
+        <v>40.887000004200004</v>
       </c>
       <c r="H8" s="2">
-        <v>0.22195352097611887</v>
+        <v>0.05548838024402972</v>
       </c>
       <c r="I8" s="2">
-        <v>0.20987954841568132</v>
+        <v>2.2687534032706944</v>
       </c>
       <c r="J8" s="2">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">945.601</t>
+          <t xml:space="preserve">1947.000</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="N8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="O8" s="0" t="inlineStr">
@@ -784,29 +784,29 @@
       </c>
       <c r="S8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution Bottom</t>
+          <t xml:space="preserve">Wire mesh B</t>
         </is>
       </c>
       <c r="U8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-C737C991D2B6</t>
+          <t xml:space="preserve">B-D6B42F9271BC</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -815,29 +815,29 @@
         </is>
       </c>
       <c r="D9" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="E9" s="2">
+        <v>11.0</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G9" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0.8878140839044755</v>
+      </c>
+      <c r="I9" s="2">
+        <v>4.882977461474615</v>
+      </c>
+      <c r="J9" s="2">
         <v>6.0</v>
       </c>
-      <c r="E9" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="F9" s="2">
-        <v>0.9440000002</v>
-      </c>
-      <c r="G9" s="2">
-        <v>4.720000001</v>
-      </c>
-      <c r="H9" s="2">
-        <v>0.22195352097611887</v>
-      </c>
-      <c r="I9" s="2">
-        <v>1.0476206192292348</v>
-      </c>
-      <c r="J9" s="2">
-        <v>3.0</v>
-      </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">944.000</t>
+          <t xml:space="preserve">500.000</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="N9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="O9" s="0" t="inlineStr">
@@ -875,12 +875,12 @@
       </c>
       <c r="S9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution Bottom</t>
+          <t xml:space="preserve">End dowel End</t>
         </is>
       </c>
       <c r="U9" s="0" t="inlineStr">
@@ -892,12 +892,12 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-EC740FDBD18C</t>
+          <t xml:space="preserve">B-DCB1303E84A9</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -906,29 +906,29 @@
         </is>
       </c>
       <c r="D10" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="E10" s="2">
-        <v>10.0</v>
+        <v>14.0</v>
       </c>
       <c r="F10" s="2">
-        <v>2.9440000002</v>
+        <v>2.9470000002</v>
       </c>
       <c r="G10" s="2">
-        <v>29.440000001999998</v>
+        <v>41.2580000028</v>
       </c>
       <c r="H10" s="2">
-        <v>0.22195352097611887</v>
+        <v>0.05548838024402972</v>
       </c>
       <c r="I10" s="2">
-        <v>6.534311657980847</v>
+        <v>2.289339592263546</v>
       </c>
       <c r="J10" s="2">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2944.000</t>
+          <t xml:space="preserve">2947.000</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="N10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="O10" s="0" t="inlineStr">
@@ -966,17 +966,17 @@
       </c>
       <c r="S10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution Bottom</t>
+          <t xml:space="preserve">Wire mesh A</t>
         </is>
       </c>
       <c r="U10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
         </is>
       </c>
     </row>
@@ -1057,12 +1057,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b0b2d59be5ac4d94</t>
+          <t xml:space="preserve">8f506f9ccecd47b9</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -1115,12 +1115,12 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0c72a96e112145ae</t>
+          <t xml:space="preserve">3ee88d218bad4e92</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -1173,12 +1173,12 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">38087d68cc244bf9</t>
+          <t xml:space="preserve">209b1f1451bc494b</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -1231,12 +1231,12 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fe997e18629474f</t>
+          <t xml:space="preserve">b7a73784dfff4380</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -1289,12 +1289,12 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7f2d50e69e54405c</t>
+          <t xml:space="preserve">4d29fbe8d98f4317</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -1347,12 +1347,12 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">18c89aaaf7374c14</t>
+          <t xml:space="preserve">7a5e75583a224190</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -1405,12 +1405,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8e866d2cce5b4b24</t>
+          <t xml:space="preserve">a39779e1cef74646</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -1463,12 +1463,12 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8bc17b93ccc5441f</t>
+          <t xml:space="preserve">fa27cf2ef8b4496b</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -1521,12 +1521,12 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">426055e57e7448cc</t>
+          <t xml:space="preserve">acb805938695432e</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -1579,12 +1579,12 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">04fb37d5ba4b4753</t>
+          <t xml:space="preserve">227f3a4985614282</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -1637,12 +1637,12 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8216183f81044f5f</t>
+          <t xml:space="preserve">4fa597d2f9f24ac0</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -1695,12 +1695,12 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3115b5de7c904027</t>
+          <t xml:space="preserve">2e84c9770e564129</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -1753,12 +1753,12 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2edd8ec7a87d43a2</t>
+          <t xml:space="preserve">008cb924e3524432</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -1811,12 +1811,12 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">274c297e7e534062</t>
+          <t xml:space="preserve">d2acbc2565c147b2</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -1869,12 +1869,12 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8206103288254875</t>
+          <t xml:space="preserve">d0dce5e38b52437e</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -1927,12 +1927,12 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">69713f2b72a644b9</t>
+          <t xml:space="preserve">ea5c781892b54ab6</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1985,12 +1985,12 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9b71b4766d8b4e68</t>
+          <t xml:space="preserve">886833c538a548bd</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -2043,12 +2043,12 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1aade593359340ac</t>
+          <t xml:space="preserve">c42ddca048e449d4</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -2101,12 +2101,12 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f45043a2bc75421d</t>
+          <t xml:space="preserve">d8be6f3f6911467c</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -2159,12 +2159,12 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5cec16b31ec8434d</t>
+          <t xml:space="preserve">45a04483751f4ddd</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -2217,12 +2217,12 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eeca9e8622124eb2</t>
+          <t xml:space="preserve">39ef79f5cbef4248</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -2275,12 +2275,12 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f3b49eb58f6b489c</t>
+          <t xml:space="preserve">087b45be91434b5a</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -2333,12 +2333,12 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">046550e068fd4b71</t>
+          <t xml:space="preserve">c3b3ad3064c64055</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -2391,12 +2391,12 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">78d4de322e004103</t>
+          <t xml:space="preserve">abf04a4d86ce46c5</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -2449,12 +2449,12 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">05ecff17bc5f4fe5</t>
+          <t xml:space="preserve">b07be946bce34710</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -2507,12 +2507,12 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">050f06ea77184b1a</t>
+          <t xml:space="preserve">58afce56cbac4c0a</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -2565,12 +2565,12 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4dd7213b60c145f1</t>
+          <t xml:space="preserve">89ea5273ac314698</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -2623,12 +2623,12 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2aec340c1bb54b89</t>
+          <t xml:space="preserve">bb361127e2804745</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -2681,12 +2681,12 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">38bfa12d7d394144</t>
+          <t xml:space="preserve">3f9dd89e06474bce</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -2739,12 +2739,12 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9e3cff1f57ee49c0</t>
+          <t xml:space="preserve">1631e9cacb69449a</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -2797,12 +2797,12 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4cdce383db7c4a33</t>
+          <t xml:space="preserve">7c03c46ea1824a53</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -2855,12 +2855,12 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fcfa1a432d1148ee</t>
+          <t xml:space="preserve">ce024c73b5a74eb5</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2913,12 +2913,12 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3f828f38e12744ec</t>
+          <t xml:space="preserve">0dbf2ed053c34b77</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2971,12 +2971,12 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">47fbd404c0cd4b52</t>
+          <t xml:space="preserve">7031c9f479244364</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -3029,12 +3029,12 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">355e83b23eff44aa</t>
+          <t xml:space="preserve">42832b4b4e084a04</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -3087,12 +3087,12 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0067c996cefc46b3</t>
+          <t xml:space="preserve">ed566059158745e1</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -3145,12 +3145,12 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b30c673fae31479c</t>
+          <t xml:space="preserve">a8136249b63c4f2c</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">51d7c62cc01e49e7</t>
+          <t xml:space="preserve">0fbd0770f92b4ccd</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -3203,12 +3203,12 @@
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">435e2ddd6c29433f</t>
+          <t xml:space="preserve">90f7b7ece99044e3</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -3261,12 +3261,12 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e679bacfa2b344bb</t>
+          <t xml:space="preserve">2a129fe3e15a4226</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -3319,12 +3319,12 @@
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e29308d2df7a468a</t>
+          <t xml:space="preserve">6994892455eb4fb1</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -3377,12 +3377,12 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e2a5e34d8484c19</t>
+          <t xml:space="preserve">853f7f006a5446b0</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1a5a4e8f3055428b</t>
+          <t xml:space="preserve">5076c17ca9bc4baa</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -3493,12 +3493,12 @@
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f19615d093b14196</t>
+          <t xml:space="preserve">e62f2b5886514268</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -3551,12 +3551,12 @@
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e6130323405b4c13</t>
+          <t xml:space="preserve">aa47a5cde1994bf4</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -3609,12 +3609,12 @@
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5383b1997a6f417c</t>
+          <t xml:space="preserve">2fb15d6aa7e34bbb</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -3667,12 +3667,12 @@
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">599cbba164644e72</t>
+          <t xml:space="preserve">21731e018c5e4f6a</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -3725,12 +3725,12 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bb13580369884dca</t>
+          <t xml:space="preserve">e078d7b8a7ae4943</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -3783,12 +3783,12 @@
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4b82e6c8d5a0467f</t>
+          <t xml:space="preserve">202db5389b274bee</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -3841,12 +3841,12 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d0a78a0a88534df6</t>
+          <t xml:space="preserve">7d3d0c2a4ef24182</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3899,12 +3899,12 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2eadbbde98d94493</t>
+          <t xml:space="preserve">12b47b9878d64c6c</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3957,12 +3957,12 @@
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a343df34f0b74594</t>
+          <t xml:space="preserve">4e694deb1f504a74</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -4015,12 +4015,12 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">95952a9b802040d9</t>
+          <t xml:space="preserve">4d35db77eae043c9</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -4073,12 +4073,12 @@
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">038960cb861a4622</t>
+          <t xml:space="preserve">3346f942294e48fe</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -4131,12 +4131,12 @@
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2b93a353ef644279</t>
+          <t xml:space="preserve">59462e0ecdec410e</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -4189,12 +4189,12 @@
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0dfa4d6864c2488f</t>
+          <t xml:space="preserve">a38d5eb1d0bc4ab4</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -4247,12 +4247,12 @@
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">90bdaf5b58ff4804</t>
+          <t xml:space="preserve">b206c072bb0542e6</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -4305,12 +4305,12 @@
     <row r="58">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">57772cfcfc424e5a</t>
+          <t xml:space="preserve">26153c8cea474e85</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -4363,12 +4363,12 @@
     <row r="59">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">505e5b645fbb4f1c</t>
+          <t xml:space="preserve">ead55bd71d9f434a</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -4421,12 +4421,12 @@
     <row r="60">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d009ca4aceca48b1</t>
+          <t xml:space="preserve">9208c312f5c94632</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -4479,12 +4479,12 @@
     <row r="61">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a38d551c22d84bd9</t>
+          <t xml:space="preserve">88a164e40e7e455b</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -4537,12 +4537,12 @@
     <row r="62">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a9acfa7d05494b8b</t>
+          <t xml:space="preserve">d2d06c90b2aa4c00</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -4595,12 +4595,12 @@
     <row r="63">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">05aaecddd9bf41cc</t>
+          <t xml:space="preserve">0fa91d5bab3d497a</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -4653,12 +4653,12 @@
     <row r="64">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">da50cec9e5494bd7</t>
+          <t xml:space="preserve">f2a0b44108ec4136</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -4711,12 +4711,12 @@
     <row r="65">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">de34b9d72a584a77</t>
+          <t xml:space="preserve">ce576d26025342c3</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -4769,12 +4769,12 @@
     <row r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">865a0e342bfe4883</t>
+          <t xml:space="preserve">75b77f612e2e40f6</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -4827,12 +4827,12 @@
     <row r="67">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9bf1b40607724649</t>
+          <t xml:space="preserve">41be0b15843140bb</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4885,12 +4885,12 @@
     <row r="68">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">373fbefcee714086</t>
+          <t xml:space="preserve">770aaecbf13d4e8a</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -4943,12 +4943,12 @@
     <row r="69">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">33b8e6cf91ff4bf3</t>
+          <t xml:space="preserve">7abf20a21c3d4701</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -5001,12 +5001,12 @@
     <row r="70">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1b76c89c3a3340dc</t>
+          <t xml:space="preserve">e0e91bef53fd4bc3</t>
         </is>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -5059,12 +5059,12 @@
     <row r="71">
       <c r="A71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5b873fac2c0c41a0</t>
+          <t xml:space="preserve">e1455b0fc8e34f38</t>
         </is>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -5117,12 +5117,12 @@
     <row r="72">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">032aa3b41d704dd8</t>
+          <t xml:space="preserve">28cbefbcf34045e6</t>
         </is>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -5175,12 +5175,12 @@
     <row r="73">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">95315eba25154c45</t>
+          <t xml:space="preserve">120c9d0f05964aa5</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -5233,12 +5233,12 @@
     <row r="74">
       <c r="A74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5b0c186638604faa</t>
+          <t xml:space="preserve">6150e98514be440b</t>
         </is>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -5291,12 +5291,12 @@
     <row r="75">
       <c r="A75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">18fdb24363f44869</t>
+          <t xml:space="preserve">f1dcb66e3de348ac</t>
         </is>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -5349,12 +5349,12 @@
     <row r="76">
       <c r="A76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8cccac46adbf4c42</t>
+          <t xml:space="preserve">5484a84732cc44d7</t>
         </is>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -5407,12 +5407,12 @@
     <row r="77">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3dee30f636684b16</t>
+          <t xml:space="preserve">361d3f30261f49d0</t>
         </is>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -5465,12 +5465,12 @@
     <row r="78">
       <c r="A78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c126e47c66504073</t>
+          <t xml:space="preserve">6caa656600af4186</t>
         </is>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -5523,12 +5523,12 @@
     <row r="79">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f5da02b56151451c</t>
+          <t xml:space="preserve">4040a3ccd2364cab</t>
         </is>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -5581,12 +5581,12 @@
     <row r="80">
       <c r="A80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7fda8b29514a4f74</t>
+          <t xml:space="preserve">fa6c7ebf091c4ada</t>
         </is>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -5639,12 +5639,12 @@
     <row r="81">
       <c r="A81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e6850615405b411d</t>
+          <t xml:space="preserve">04a52c596a3441d0</t>
         </is>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -5697,12 +5697,12 @@
     <row r="82">
       <c r="A82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">465730f1abd44143</t>
+          <t xml:space="preserve">cf4f17d27e284492</t>
         </is>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -5755,12 +5755,12 @@
     <row r="83">
       <c r="A83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">dd58d5a648124d7b</t>
+          <t xml:space="preserve">8720e93d4249432f</t>
         </is>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -5813,12 +5813,12 @@
     <row r="84">
       <c r="A84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6305aa2d1c504d29</t>
+          <t xml:space="preserve">32055e50c34e4b50</t>
         </is>
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -5871,12 +5871,12 @@
     <row r="85">
       <c r="A85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">72da5a95fe5e407d</t>
+          <t xml:space="preserve">b0d1f091e0904ab1</t>
         </is>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -5929,12 +5929,12 @@
     <row r="86">
       <c r="A86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">53d8193e88624e07</t>
+          <t xml:space="preserve">bc427587896d45dd</t>
         </is>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -5987,12 +5987,12 @@
     <row r="87">
       <c r="A87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">80bef32ca9474d0b</t>
+          <t xml:space="preserve">f074b96b66df4be6</t>
         </is>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -6045,12 +6045,12 @@
     <row r="88">
       <c r="A88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e344713a51a4d85</t>
+          <t xml:space="preserve">41454c8f5a854918</t>
         </is>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -6103,12 +6103,12 @@
     <row r="89">
       <c r="A89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">454cb8cb49cd4600</t>
+          <t xml:space="preserve">9925001ca0ae4c01</t>
         </is>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -6161,12 +6161,12 @@
     <row r="90">
       <c r="A90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">665f685cfefa4c50</t>
+          <t xml:space="preserve">5b92034f1ff2418d</t>
         </is>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -6219,12 +6219,12 @@
     <row r="91">
       <c r="A91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ded3bc351f0f4063</t>
+          <t xml:space="preserve">151a3ae4e62c406c</t>
         </is>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -6277,12 +6277,12 @@
     <row r="92">
       <c r="A92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b410e0988c9c4346</t>
+          <t xml:space="preserve">ebc7594d9726410e</t>
         </is>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -6335,12 +6335,12 @@
     <row r="93">
       <c r="A93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">45ea11626aab4c42</t>
+          <t xml:space="preserve">946795dfede44a01</t>
         </is>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -6393,12 +6393,12 @@
     <row r="94">
       <c r="A94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">915fe051f7c94022</t>
+          <t xml:space="preserve">7126ca0af62d41b5</t>
         </is>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -6451,12 +6451,12 @@
     <row r="95">
       <c r="A95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9d94b5ef77a94e62</t>
+          <t xml:space="preserve">2cc068c31d554ca1</t>
         </is>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">37159d2f5d2e42df</t>
+          <t xml:space="preserve">eb41e416dedf46d1</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Add project RC stair type library and immutable instance snapshots
</commit_message>
<xml_diff>
--- a/examples/extensions/thai_bim/examples/slab-reinforcement-BBS.xlsx
+++ b/examples/extensions/thai_bim/examples/slab-reinforcement-BBS.xlsx
@@ -213,7 +213,7 @@
       </c>
       <c r="N2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="O2" s="0" t="inlineStr">
@@ -304,7 +304,7 @@
       </c>
       <c r="N3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="O3" s="0" t="inlineStr">
@@ -395,7 +395,7 @@
       </c>
       <c r="N4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="O4" s="0" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="N5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="O5" s="0" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="N6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="O6" s="0" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="N7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="O7" s="0" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="N8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="O8" s="0" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="N9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="O9" s="0" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="N10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="O10" s="0" t="inlineStr">
@@ -1057,12 +1057,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8f506f9ccecd47b9</t>
+          <t xml:space="preserve">20c13fb158f1432d</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -1115,12 +1115,12 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3ee88d218bad4e92</t>
+          <t xml:space="preserve">650cdaf37f30453c</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -1173,12 +1173,12 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">209b1f1451bc494b</t>
+          <t xml:space="preserve">fbddec3ef1b6490b</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -1231,12 +1231,12 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b7a73784dfff4380</t>
+          <t xml:space="preserve">e3a345df49d24ebd</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -1289,12 +1289,12 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4d29fbe8d98f4317</t>
+          <t xml:space="preserve">5a11f69b50d64ee7</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -1347,12 +1347,12 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7a5e75583a224190</t>
+          <t xml:space="preserve">7931a1f4d966428d</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -1405,12 +1405,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a39779e1cef74646</t>
+          <t xml:space="preserve">b075504c187c44c1</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -1463,12 +1463,12 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fa27cf2ef8b4496b</t>
+          <t xml:space="preserve">c9d955727bba4aea</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -1521,12 +1521,12 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">acb805938695432e</t>
+          <t xml:space="preserve">7db1a0a74db94c49</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -1579,12 +1579,12 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">227f3a4985614282</t>
+          <t xml:space="preserve">74e4c85ffe5d4fd7</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -1637,12 +1637,12 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4fa597d2f9f24ac0</t>
+          <t xml:space="preserve">611eb07c1243496e</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -1695,12 +1695,12 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2e84c9770e564129</t>
+          <t xml:space="preserve">93fabf73df004250</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -1753,12 +1753,12 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">008cb924e3524432</t>
+          <t xml:space="preserve">9e8eec0d19664d39</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -1811,12 +1811,12 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d2acbc2565c147b2</t>
+          <t xml:space="preserve">cb0df2c92a764550</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -1869,12 +1869,12 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d0dce5e38b52437e</t>
+          <t xml:space="preserve">4e93da06b483450d</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -1927,12 +1927,12 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ea5c781892b54ab6</t>
+          <t xml:space="preserve">89fbd728bb5c41b0</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1985,12 +1985,12 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">886833c538a548bd</t>
+          <t xml:space="preserve">3fb778994dae454e</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -2043,12 +2043,12 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c42ddca048e449d4</t>
+          <t xml:space="preserve">b64b4b6b2b044ca3</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -2101,12 +2101,12 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d8be6f3f6911467c</t>
+          <t xml:space="preserve">83479672e22845d5</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -2159,12 +2159,12 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">45a04483751f4ddd</t>
+          <t xml:space="preserve">9d038e8ed77f44c7</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -2217,12 +2217,12 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">39ef79f5cbef4248</t>
+          <t xml:space="preserve">d66b3820127b41a3</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -2275,12 +2275,12 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">087b45be91434b5a</t>
+          <t xml:space="preserve">b7c355aa167740c9</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -2333,12 +2333,12 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c3b3ad3064c64055</t>
+          <t xml:space="preserve">6c176a7386f44b08</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -2391,12 +2391,12 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">abf04a4d86ce46c5</t>
+          <t xml:space="preserve">4ae9a0b610394536</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -2449,12 +2449,12 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b07be946bce34710</t>
+          <t xml:space="preserve">40cdc20d16c34c8b</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -2507,12 +2507,12 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">58afce56cbac4c0a</t>
+          <t xml:space="preserve">849de5f700cb4a2e</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -2565,12 +2565,12 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">89ea5273ac314698</t>
+          <t xml:space="preserve">d891eee18c474f23</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -2623,12 +2623,12 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bb361127e2804745</t>
+          <t xml:space="preserve">36b6b42c426e412a</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -2681,12 +2681,12 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3f9dd89e06474bce</t>
+          <t xml:space="preserve">d70e8ba5476346fb</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -2739,12 +2739,12 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1631e9cacb69449a</t>
+          <t xml:space="preserve">bfb1bb00c91b4348</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -2797,12 +2797,12 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7c03c46ea1824a53</t>
+          <t xml:space="preserve">3af7583138424562</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -2855,12 +2855,12 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ce024c73b5a74eb5</t>
+          <t xml:space="preserve">a7a45611de124d8a</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2913,12 +2913,12 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0dbf2ed053c34b77</t>
+          <t xml:space="preserve">1efc9fdfc24b4688</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2971,12 +2971,12 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7031c9f479244364</t>
+          <t xml:space="preserve">822e99e88e244bfb</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -3029,12 +3029,12 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">42832b4b4e084a04</t>
+          <t xml:space="preserve">3e7675294d7f4631</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -3087,12 +3087,12 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ed566059158745e1</t>
+          <t xml:space="preserve">98c937de2cf84e90</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -3145,12 +3145,12 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a8136249b63c4f2c</t>
+          <t xml:space="preserve">c9eaaff8ac634de9</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fbd0770f92b4ccd</t>
+          <t xml:space="preserve">860c9984e57d4854</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -3203,12 +3203,12 @@
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">90f7b7ece99044e3</t>
+          <t xml:space="preserve">658a41e15fbd49d3</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -3261,12 +3261,12 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2a129fe3e15a4226</t>
+          <t xml:space="preserve">d77fa86f99f7484d</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -3319,12 +3319,12 @@
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6994892455eb4fb1</t>
+          <t xml:space="preserve">2e945bca29354f20</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -3377,12 +3377,12 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">853f7f006a5446b0</t>
+          <t xml:space="preserve">0917f798ec2a4358</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5076c17ca9bc4baa</t>
+          <t xml:space="preserve">99569aee111d40df</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -3493,12 +3493,12 @@
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e62f2b5886514268</t>
+          <t xml:space="preserve">92a4454b87444e4c</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -3551,12 +3551,12 @@
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aa47a5cde1994bf4</t>
+          <t xml:space="preserve">7470ed34b5084b8e</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -3609,12 +3609,12 @@
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2fb15d6aa7e34bbb</t>
+          <t xml:space="preserve">bf1fda7ff5534ee4</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -3667,12 +3667,12 @@
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">21731e018c5e4f6a</t>
+          <t xml:space="preserve">9616865aa2b24e0d</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -3725,12 +3725,12 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e078d7b8a7ae4943</t>
+          <t xml:space="preserve">98a9a8fb28604513</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -3783,12 +3783,12 @@
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">202db5389b274bee</t>
+          <t xml:space="preserve">0767f2dfc7dd4792</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -3841,12 +3841,12 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7d3d0c2a4ef24182</t>
+          <t xml:space="preserve">77cdae5f99fc4d12</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3899,12 +3899,12 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">12b47b9878d64c6c</t>
+          <t xml:space="preserve">f43b423b4e3f464b</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3957,12 +3957,12 @@
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4e694deb1f504a74</t>
+          <t xml:space="preserve">cb4d355205a74b77</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -4015,12 +4015,12 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4d35db77eae043c9</t>
+          <t xml:space="preserve">2befcb7d7bf945c1</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -4073,12 +4073,12 @@
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3346f942294e48fe</t>
+          <t xml:space="preserve">d173be788493497b</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -4131,12 +4131,12 @@
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">59462e0ecdec410e</t>
+          <t xml:space="preserve">dac830d5e4454f67</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -4189,12 +4189,12 @@
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a38d5eb1d0bc4ab4</t>
+          <t xml:space="preserve">3ea4e4024f5f4e75</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -4247,12 +4247,12 @@
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b206c072bb0542e6</t>
+          <t xml:space="preserve">379e1854963e4cb1</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -4305,12 +4305,12 @@
     <row r="58">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">26153c8cea474e85</t>
+          <t xml:space="preserve">3324146c7ba8454c</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -4363,12 +4363,12 @@
     <row r="59">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ead55bd71d9f434a</t>
+          <t xml:space="preserve">d48b7bd132594eed</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -4421,12 +4421,12 @@
     <row r="60">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9208c312f5c94632</t>
+          <t xml:space="preserve">2eb1715ad62e42e9</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -4479,12 +4479,12 @@
     <row r="61">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">88a164e40e7e455b</t>
+          <t xml:space="preserve">ad85e92407cf4295</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -4537,12 +4537,12 @@
     <row r="62">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d2d06c90b2aa4c00</t>
+          <t xml:space="preserve">675190652d3f44c1</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -4595,12 +4595,12 @@
     <row r="63">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fa91d5bab3d497a</t>
+          <t xml:space="preserve">001790d8cef94ffd</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -4653,12 +4653,12 @@
     <row r="64">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f2a0b44108ec4136</t>
+          <t xml:space="preserve">c2a7aaeff3cf458d</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -4711,12 +4711,12 @@
     <row r="65">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ce576d26025342c3</t>
+          <t xml:space="preserve">a95a2b5d6de44a3b</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -4769,12 +4769,12 @@
     <row r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">75b77f612e2e40f6</t>
+          <t xml:space="preserve">00744b49b26145de</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -4827,12 +4827,12 @@
     <row r="67">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">41be0b15843140bb</t>
+          <t xml:space="preserve">f11d66b62b2b4afd</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4885,12 +4885,12 @@
     <row r="68">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">770aaecbf13d4e8a</t>
+          <t xml:space="preserve">59f38649d74d4368</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -4943,12 +4943,12 @@
     <row r="69">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7abf20a21c3d4701</t>
+          <t xml:space="preserve">bee2280453b94cfc</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -5001,12 +5001,12 @@
     <row r="70">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e0e91bef53fd4bc3</t>
+          <t xml:space="preserve">bb843da7325e401c</t>
         </is>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -5059,12 +5059,12 @@
     <row r="71">
       <c r="A71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e1455b0fc8e34f38</t>
+          <t xml:space="preserve">eb89032ac49c49c1</t>
         </is>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -5117,12 +5117,12 @@
     <row r="72">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">28cbefbcf34045e6</t>
+          <t xml:space="preserve">bf970f255f3740f5</t>
         </is>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -5175,12 +5175,12 @@
     <row r="73">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">120c9d0f05964aa5</t>
+          <t xml:space="preserve">6559319ffe5f44fc</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -5233,12 +5233,12 @@
     <row r="74">
       <c r="A74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6150e98514be440b</t>
+          <t xml:space="preserve">419f3351d18249de</t>
         </is>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -5291,12 +5291,12 @@
     <row r="75">
       <c r="A75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f1dcb66e3de348ac</t>
+          <t xml:space="preserve">963f86e3ad254474</t>
         </is>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -5349,12 +5349,12 @@
     <row r="76">
       <c r="A76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5484a84732cc44d7</t>
+          <t xml:space="preserve">389b677ffa0d46c8</t>
         </is>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -5407,12 +5407,12 @@
     <row r="77">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">361d3f30261f49d0</t>
+          <t xml:space="preserve">6d92cb51672040f8</t>
         </is>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -5465,12 +5465,12 @@
     <row r="78">
       <c r="A78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6caa656600af4186</t>
+          <t xml:space="preserve">cba8f8d3f90f4d21</t>
         </is>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -5523,12 +5523,12 @@
     <row r="79">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4040a3ccd2364cab</t>
+          <t xml:space="preserve">081eeb6d27fc4a52</t>
         </is>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -5581,12 +5581,12 @@
     <row r="80">
       <c r="A80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fa6c7ebf091c4ada</t>
+          <t xml:space="preserve">b3e9a9ce9e004bb2</t>
         </is>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -5639,12 +5639,12 @@
     <row r="81">
       <c r="A81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">04a52c596a3441d0</t>
+          <t xml:space="preserve">ae53055f16aa4333</t>
         </is>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -5697,12 +5697,12 @@
     <row r="82">
       <c r="A82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cf4f17d27e284492</t>
+          <t xml:space="preserve">c0c9ceb295e240c0</t>
         </is>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -5755,12 +5755,12 @@
     <row r="83">
       <c r="A83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8720e93d4249432f</t>
+          <t xml:space="preserve">d6a32fb5ed884e78</t>
         </is>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -5813,12 +5813,12 @@
     <row r="84">
       <c r="A84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">32055e50c34e4b50</t>
+          <t xml:space="preserve">fb1e78a659054806</t>
         </is>
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -5871,12 +5871,12 @@
     <row r="85">
       <c r="A85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b0d1f091e0904ab1</t>
+          <t xml:space="preserve">f133936cc9324cbb</t>
         </is>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -5929,12 +5929,12 @@
     <row r="86">
       <c r="A86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bc427587896d45dd</t>
+          <t xml:space="preserve">1e5f2ca5746747ab</t>
         </is>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -5987,12 +5987,12 @@
     <row r="87">
       <c r="A87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f074b96b66df4be6</t>
+          <t xml:space="preserve">12f2c21addcc4287</t>
         </is>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -6045,12 +6045,12 @@
     <row r="88">
       <c r="A88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">41454c8f5a854918</t>
+          <t xml:space="preserve">02295b9817fe43ac</t>
         </is>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -6103,12 +6103,12 @@
     <row r="89">
       <c r="A89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9925001ca0ae4c01</t>
+          <t xml:space="preserve">61cd8dc953914e2a</t>
         </is>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -6161,12 +6161,12 @@
     <row r="90">
       <c r="A90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5b92034f1ff2418d</t>
+          <t xml:space="preserve">d3017c8a1e3542cd</t>
         </is>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -6219,12 +6219,12 @@
     <row r="91">
       <c r="A91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">151a3ae4e62c406c</t>
+          <t xml:space="preserve">672ed99b172c4955</t>
         </is>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -6277,12 +6277,12 @@
     <row r="92">
       <c r="A92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ebc7594d9726410e</t>
+          <t xml:space="preserve">3f89ad08e0864e1d</t>
         </is>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -6335,12 +6335,12 @@
     <row r="93">
       <c r="A93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">946795dfede44a01</t>
+          <t xml:space="preserve">f661327d1e354a0a</t>
         </is>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -6393,12 +6393,12 @@
     <row r="94">
       <c r="A94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7126ca0af62d41b5</t>
+          <t xml:space="preserve">ba8fc7598c794284</t>
         </is>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -6451,12 +6451,12 @@
     <row r="95">
       <c r="A95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2cc068c31d554ca1</t>
+          <t xml:space="preserve">c63aa8a8e7af4636</t>
         </is>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb41e416dedf46d1</t>
+          <t xml:space="preserve">e295f92f55be4af5</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Add native two-point snap placement for all RC stair forms
</commit_message>
<xml_diff>
--- a/examples/extensions/thai_bim/examples/slab-reinforcement-BBS.xlsx
+++ b/examples/extensions/thai_bim/examples/slab-reinforcement-BBS.xlsx
@@ -164,12 +164,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-4068504360E9</t>
+          <t xml:space="preserve">B-4E26E3FCA12B</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -181,26 +181,26 @@
         <v>12.0</v>
       </c>
       <c r="E2" s="2">
-        <v>7.0</v>
+        <v>11.0</v>
       </c>
       <c r="F2" s="2">
-        <v>2.9380000001999997</v>
+        <v>0.5</v>
       </c>
       <c r="G2" s="2">
-        <v>20.5660000014</v>
+        <v>5.5</v>
       </c>
       <c r="H2" s="2">
         <v>0.8878140839044755</v>
       </c>
       <c r="I2" s="2">
-        <v>18.258784450822382</v>
+        <v>4.882977461474615</v>
       </c>
       <c r="J2" s="2">
         <v>6.0</v>
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2938.000</t>
+          <t xml:space="preserve">500.000</t>
         </is>
       </c>
       <c r="L2" s="0" t="inlineStr">
@@ -213,7 +213,7 @@
       </c>
       <c r="N2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="O2" s="0" t="inlineStr">
@@ -238,12 +238,12 @@
       </c>
       <c r="S2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main Bottom</t>
+          <t xml:space="preserve">End dowel Start</t>
         </is>
       </c>
       <c r="U2" s="0" t="inlineStr">
@@ -255,12 +255,12 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-54ED5FEFBD3F</t>
+          <t xml:space="preserve">B-A359E7AF0105</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -269,29 +269,29 @@
         </is>
       </c>
       <c r="D3" s="2">
-        <v>12.0</v>
+        <v>3.0</v>
       </c>
       <c r="E3" s="2">
-        <v>14.0</v>
+        <v>21.0</v>
       </c>
       <c r="F3" s="2">
-        <v>1.9380000002</v>
+        <v>1.9470000002</v>
       </c>
       <c r="G3" s="2">
-        <v>27.132000002799998</v>
+        <v>40.887000004200004</v>
       </c>
       <c r="H3" s="2">
-        <v>0.8878140839044755</v>
+        <v>0.05548838024402972</v>
       </c>
       <c r="I3" s="2">
-        <v>24.08817172698211</v>
+        <v>2.2687534032706944</v>
       </c>
       <c r="J3" s="2">
-        <v>6.0</v>
+        <v>1.5</v>
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1938.000</t>
+          <t xml:space="preserve">1947.000</t>
         </is>
       </c>
       <c r="L3" s="0" t="inlineStr">
@@ -304,7 +304,7 @@
       </c>
       <c r="N3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="O3" s="0" t="inlineStr">
@@ -329,29 +329,29 @@
       </c>
       <c r="S3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main Bottom</t>
+          <t xml:space="preserve">Wire mesh B</t>
         </is>
       </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-74C88A2DAA56</t>
+          <t xml:space="preserve">B-D6B42F9271BC</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -360,29 +360,29 @@
         </is>
       </c>
       <c r="D4" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>11.0</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G4" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.8878140839044755</v>
+      </c>
+      <c r="I4" s="2">
+        <v>4.882977461474615</v>
+      </c>
+      <c r="J4" s="2">
         <v>6.0</v>
       </c>
-      <c r="E4" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0.9456013470417681</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0.9456013470417681</v>
-      </c>
-      <c r="H4" s="2">
-        <v>0.22195352097611887</v>
-      </c>
-      <c r="I4" s="2">
-        <v>0.20987954841568132</v>
-      </c>
-      <c r="J4" s="2">
-        <v>3.0</v>
-      </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">945.601</t>
+          <t xml:space="preserve">500.000</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
@@ -395,7 +395,7 @@
       </c>
       <c r="N4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="O4" s="0" t="inlineStr">
@@ -420,12 +420,12 @@
       </c>
       <c r="S4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution Bottom</t>
+          <t xml:space="preserve">End dowel End</t>
         </is>
       </c>
       <c r="U4" s="0" t="inlineStr">
@@ -437,12 +437,12 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-C737C991D2B6</t>
+          <t xml:space="preserve">B-DCB1303E84A9</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -451,29 +451,29 @@
         </is>
       </c>
       <c r="D5" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="E5" s="2">
-        <v>5.0</v>
+        <v>14.0</v>
       </c>
       <c r="F5" s="2">
-        <v>0.9440000002</v>
+        <v>2.9470000002</v>
       </c>
       <c r="G5" s="2">
-        <v>4.720000001</v>
+        <v>41.2580000028</v>
       </c>
       <c r="H5" s="2">
-        <v>0.22195352097611887</v>
+        <v>0.05548838024402972</v>
       </c>
       <c r="I5" s="2">
-        <v>1.0476206192292348</v>
+        <v>2.289339592263546</v>
       </c>
       <c r="J5" s="2">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">944.000</t>
+          <t xml:space="preserve">2947.000</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="N5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="O5" s="0" t="inlineStr">
@@ -511,17 +511,17 @@
       </c>
       <c r="S5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution Bottom</t>
+          <t xml:space="preserve">Wire mesh A</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-EC740FDBD18C</t>
+          <t xml:space="preserve">B-4068504360E9</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -542,29 +542,29 @@
         </is>
       </c>
       <c r="D6" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>2.9380000001999997</v>
+      </c>
+      <c r="G6" s="2">
+        <v>20.5660000014</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0.8878140839044755</v>
+      </c>
+      <c r="I6" s="2">
+        <v>18.258784450822382</v>
+      </c>
+      <c r="J6" s="2">
         <v>6.0</v>
       </c>
-      <c r="E6" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="F6" s="2">
-        <v>2.9440000002</v>
-      </c>
-      <c r="G6" s="2">
-        <v>29.440000001999998</v>
-      </c>
-      <c r="H6" s="2">
-        <v>0.22195352097611887</v>
-      </c>
-      <c r="I6" s="2">
-        <v>6.534311657980847</v>
-      </c>
-      <c r="J6" s="2">
-        <v>3.0</v>
-      </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2944.000</t>
+          <t xml:space="preserve">2938.000</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="N6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="O6" s="0" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="T6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution Bottom</t>
+          <t xml:space="preserve">Main Bottom</t>
         </is>
       </c>
       <c r="U6" s="0" t="inlineStr">
@@ -619,12 +619,12 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-4E26E3FCA12B</t>
+          <t xml:space="preserve">B-54ED5FEFBD3F</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -636,26 +636,26 @@
         <v>12.0</v>
       </c>
       <c r="E7" s="2">
-        <v>11.0</v>
+        <v>14.0</v>
       </c>
       <c r="F7" s="2">
-        <v>0.5</v>
+        <v>1.9380000002</v>
       </c>
       <c r="G7" s="2">
-        <v>5.5</v>
+        <v>27.132000002799998</v>
       </c>
       <c r="H7" s="2">
         <v>0.8878140839044755</v>
       </c>
       <c r="I7" s="2">
-        <v>4.882977461474615</v>
+        <v>24.08817172698211</v>
       </c>
       <c r="J7" s="2">
         <v>6.0</v>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">500.000</t>
+          <t xml:space="preserve">1938.000</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="N7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="O7" s="0" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="S7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">End dowel Start</t>
+          <t xml:space="preserve">Main Bottom</t>
         </is>
       </c>
       <c r="U7" s="0" t="inlineStr">
@@ -710,12 +710,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-A359E7AF0105</t>
+          <t xml:space="preserve">B-74C88A2DAA56</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -724,29 +724,29 @@
         </is>
       </c>
       <c r="D8" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.9456013470417681</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.9456013470417681</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0.22195352097611887</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0.20987954841568132</v>
+      </c>
+      <c r="J8" s="2">
         <v>3.0</v>
       </c>
-      <c r="E8" s="2">
-        <v>21.0</v>
-      </c>
-      <c r="F8" s="2">
-        <v>1.9470000002</v>
-      </c>
-      <c r="G8" s="2">
-        <v>40.887000004200004</v>
-      </c>
-      <c r="H8" s="2">
-        <v>0.05548838024402972</v>
-      </c>
-      <c r="I8" s="2">
-        <v>2.2687534032706944</v>
-      </c>
-      <c r="J8" s="2">
-        <v>1.5</v>
-      </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1947.000</t>
+          <t xml:space="preserve">945.601</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="N8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="O8" s="0" t="inlineStr">
@@ -784,29 +784,29 @@
       </c>
       <c r="S8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wire mesh B</t>
+          <t xml:space="preserve">Distribution Bottom</t>
         </is>
       </c>
       <c r="U8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-D6B42F9271BC</t>
+          <t xml:space="preserve">B-C737C991D2B6</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -815,29 +815,29 @@
         </is>
       </c>
       <c r="D9" s="2">
-        <v>12.0</v>
+        <v>6.0</v>
       </c>
       <c r="E9" s="2">
-        <v>11.0</v>
+        <v>5.0</v>
       </c>
       <c r="F9" s="2">
-        <v>0.5</v>
+        <v>0.9440000002</v>
       </c>
       <c r="G9" s="2">
-        <v>5.5</v>
+        <v>4.720000001</v>
       </c>
       <c r="H9" s="2">
-        <v>0.8878140839044755</v>
+        <v>0.22195352097611887</v>
       </c>
       <c r="I9" s="2">
-        <v>4.882977461474615</v>
+        <v>1.0476206192292348</v>
       </c>
       <c r="J9" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">500.000</t>
+          <t xml:space="preserve">944.000</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="N9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="O9" s="0" t="inlineStr">
@@ -875,12 +875,12 @@
       </c>
       <c r="S9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">End dowel End</t>
+          <t xml:space="preserve">Distribution Bottom</t>
         </is>
       </c>
       <c r="U9" s="0" t="inlineStr">
@@ -892,12 +892,12 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-DCB1303E84A9</t>
+          <t xml:space="preserve">B-EC740FDBD18C</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -906,29 +906,29 @@
         </is>
       </c>
       <c r="D10" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="E10" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="F10" s="2">
+        <v>2.9440000002</v>
+      </c>
+      <c r="G10" s="2">
+        <v>29.440000001999998</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0.22195352097611887</v>
+      </c>
+      <c r="I10" s="2">
+        <v>6.534311657980847</v>
+      </c>
+      <c r="J10" s="2">
         <v>3.0</v>
       </c>
-      <c r="E10" s="2">
-        <v>14.0</v>
-      </c>
-      <c r="F10" s="2">
-        <v>2.9470000002</v>
-      </c>
-      <c r="G10" s="2">
-        <v>41.2580000028</v>
-      </c>
-      <c r="H10" s="2">
-        <v>0.05548838024402972</v>
-      </c>
-      <c r="I10" s="2">
-        <v>2.289339592263546</v>
-      </c>
-      <c r="J10" s="2">
-        <v>1.5</v>
-      </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2947.000</t>
+          <t xml:space="preserve">2944.000</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="N10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="O10" s="0" t="inlineStr">
@@ -966,17 +966,17 @@
       </c>
       <c r="S10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wire mesh A</t>
+          <t xml:space="preserve">Distribution Bottom</t>
         </is>
       </c>
       <c r="U10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -1057,12 +1057,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">20c13fb158f1432d</t>
+          <t xml:space="preserve">0d796e43a5dc458c</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -1115,12 +1115,12 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">650cdaf37f30453c</t>
+          <t xml:space="preserve">d2bf9e94e149462f</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -1173,12 +1173,12 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fbddec3ef1b6490b</t>
+          <t xml:space="preserve">2463f9bd593e425f</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -1231,12 +1231,12 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3a345df49d24ebd</t>
+          <t xml:space="preserve">95ae9e30887d416a</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -1289,12 +1289,12 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5a11f69b50d64ee7</t>
+          <t xml:space="preserve">b7b224d81f3a4258</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -1347,12 +1347,12 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7931a1f4d966428d</t>
+          <t xml:space="preserve">8a15ddd650264220</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -1405,12 +1405,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b075504c187c44c1</t>
+          <t xml:space="preserve">da5bec25e7484abc</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -1463,12 +1463,12 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c9d955727bba4aea</t>
+          <t xml:space="preserve">666118299db946b9</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -1521,12 +1521,12 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7db1a0a74db94c49</t>
+          <t xml:space="preserve">2fd40d8896a146c4</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -1579,12 +1579,12 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">74e4c85ffe5d4fd7</t>
+          <t xml:space="preserve">e15111740c9f4bfa</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -1637,12 +1637,12 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">611eb07c1243496e</t>
+          <t xml:space="preserve">01c49070802540e3</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -1695,12 +1695,12 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">93fabf73df004250</t>
+          <t xml:space="preserve">2e73926c88274f2d</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -1753,12 +1753,12 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9e8eec0d19664d39</t>
+          <t xml:space="preserve">1afa20a805014b9a</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -1811,12 +1811,12 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cb0df2c92a764550</t>
+          <t xml:space="preserve">4ca389f43f9040c2</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -1869,12 +1869,12 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4e93da06b483450d</t>
+          <t xml:space="preserve">80e6dcda1d6d496a</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -1927,12 +1927,12 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">89fbd728bb5c41b0</t>
+          <t xml:space="preserve">dcb9d2742559441b</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1985,12 +1985,12 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3fb778994dae454e</t>
+          <t xml:space="preserve">f9c59b4086ed490b</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -2043,12 +2043,12 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b64b4b6b2b044ca3</t>
+          <t xml:space="preserve">3d5f6aa53b46474f</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -2101,12 +2101,12 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">83479672e22845d5</t>
+          <t xml:space="preserve">375ac762864d433a</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -2159,12 +2159,12 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9d038e8ed77f44c7</t>
+          <t xml:space="preserve">a1573a96c8894b04</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -2217,12 +2217,12 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d66b3820127b41a3</t>
+          <t xml:space="preserve">d663efbf22464951</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -2275,12 +2275,12 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b7c355aa167740c9</t>
+          <t xml:space="preserve">15c1c4e0d1fb43c1</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -2333,12 +2333,12 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6c176a7386f44b08</t>
+          <t xml:space="preserve">342a50776f01483c</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -2391,12 +2391,12 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4ae9a0b610394536</t>
+          <t xml:space="preserve">58b7fa1ca7d74f65</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -2449,12 +2449,12 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">40cdc20d16c34c8b</t>
+          <t xml:space="preserve">fc7e2015960d47ce</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -2507,12 +2507,12 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">849de5f700cb4a2e</t>
+          <t xml:space="preserve">bac15b3a3f45440b</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -2565,12 +2565,12 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d891eee18c474f23</t>
+          <t xml:space="preserve">188d0989beff4d65</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -2623,12 +2623,12 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">36b6b42c426e412a</t>
+          <t xml:space="preserve">112cb946752340a5</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -2681,12 +2681,12 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d70e8ba5476346fb</t>
+          <t xml:space="preserve">90ef75e0bbfe4424</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -2739,12 +2739,12 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bfb1bb00c91b4348</t>
+          <t xml:space="preserve">601ddae8e63944e8</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -2797,12 +2797,12 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3af7583138424562</t>
+          <t xml:space="preserve">5f735eea602f4ff7</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -2855,12 +2855,12 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a7a45611de124d8a</t>
+          <t xml:space="preserve">e8a5efc1e62f4f5e</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2913,12 +2913,12 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1efc9fdfc24b4688</t>
+          <t xml:space="preserve">bb6be0baa44343d9</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2971,12 +2971,12 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">822e99e88e244bfb</t>
+          <t xml:space="preserve">c94c8dc519704290</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -3029,12 +3029,12 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3e7675294d7f4631</t>
+          <t xml:space="preserve">c9ceb61d59e24a0c</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -3087,12 +3087,12 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">98c937de2cf84e90</t>
+          <t xml:space="preserve">40a5c132c8454804</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -3145,12 +3145,12 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c9eaaff8ac634de9</t>
+          <t xml:space="preserve">0e72cbc6fc6f4758</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">860c9984e57d4854</t>
+          <t xml:space="preserve">ac69a8dd966845d7</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -3203,12 +3203,12 @@
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">658a41e15fbd49d3</t>
+          <t xml:space="preserve">3ec414a1b88845e7</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -3261,12 +3261,12 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d77fa86f99f7484d</t>
+          <t xml:space="preserve">aa225fbc2c0644e3</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -3319,12 +3319,12 @@
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2e945bca29354f20</t>
+          <t xml:space="preserve">a5601e68369747b5</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -3377,12 +3377,12 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0917f798ec2a4358</t>
+          <t xml:space="preserve">307743a2f46c4f6c</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">99569aee111d40df</t>
+          <t xml:space="preserve">bad7b266ed77445f</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -3493,12 +3493,12 @@
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">92a4454b87444e4c</t>
+          <t xml:space="preserve">2ff59de791ae4b7b</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -3551,12 +3551,12 @@
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7470ed34b5084b8e</t>
+          <t xml:space="preserve">db8d8a8c24dd42ec</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -3609,12 +3609,12 @@
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bf1fda7ff5534ee4</t>
+          <t xml:space="preserve">5a052fb081c34077</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -3667,12 +3667,12 @@
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9616865aa2b24e0d</t>
+          <t xml:space="preserve">405a417046d24628</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -3725,12 +3725,12 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">98a9a8fb28604513</t>
+          <t xml:space="preserve">1870a730ffa54191</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -3783,12 +3783,12 @@
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0767f2dfc7dd4792</t>
+          <t xml:space="preserve">e6e90c1461d74666</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -3841,12 +3841,12 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">77cdae5f99fc4d12</t>
+          <t xml:space="preserve">416df7a6e20848ab</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3899,12 +3899,12 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f43b423b4e3f464b</t>
+          <t xml:space="preserve">f0687d49f0674176</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3957,12 +3957,12 @@
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cb4d355205a74b77</t>
+          <t xml:space="preserve">f62c5ed57d2e4dee</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -4015,12 +4015,12 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2befcb7d7bf945c1</t>
+          <t xml:space="preserve">4092b0cf9d3f4564</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -4073,12 +4073,12 @@
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d173be788493497b</t>
+          <t xml:space="preserve">a4efe3896afe4fef</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -4131,12 +4131,12 @@
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">dac830d5e4454f67</t>
+          <t xml:space="preserve">41ac9eb7e5cc4e5a</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -4189,12 +4189,12 @@
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3ea4e4024f5f4e75</t>
+          <t xml:space="preserve">76bbb129bfe4415c</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -4247,12 +4247,12 @@
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">379e1854963e4cb1</t>
+          <t xml:space="preserve">88801c1f42e646e1</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -4305,12 +4305,12 @@
     <row r="58">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3324146c7ba8454c</t>
+          <t xml:space="preserve">5be36060bb6f483b</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -4363,12 +4363,12 @@
     <row r="59">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d48b7bd132594eed</t>
+          <t xml:space="preserve">aac1760efebf4d1c</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -4421,12 +4421,12 @@
     <row r="60">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2eb1715ad62e42e9</t>
+          <t xml:space="preserve">e69b1fcc4ee34039</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -4479,12 +4479,12 @@
     <row r="61">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ad85e92407cf4295</t>
+          <t xml:space="preserve">90de4dc1c46b449d</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -4537,12 +4537,12 @@
     <row r="62">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">675190652d3f44c1</t>
+          <t xml:space="preserve">603832b5897b488d</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -4595,12 +4595,12 @@
     <row r="63">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">001790d8cef94ffd</t>
+          <t xml:space="preserve">1900ba1079c34ecf</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -4653,12 +4653,12 @@
     <row r="64">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c2a7aaeff3cf458d</t>
+          <t xml:space="preserve">a68e9c0dc0bd46c2</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -4711,12 +4711,12 @@
     <row r="65">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a95a2b5d6de44a3b</t>
+          <t xml:space="preserve">e40399b122a94226</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -4769,12 +4769,12 @@
     <row r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">00744b49b26145de</t>
+          <t xml:space="preserve">89efea1cf8b24b09</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -4827,12 +4827,12 @@
     <row r="67">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f11d66b62b2b4afd</t>
+          <t xml:space="preserve">d305baf593384870</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4885,12 +4885,12 @@
     <row r="68">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">59f38649d74d4368</t>
+          <t xml:space="preserve">fe712f03b99843a1</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -4943,12 +4943,12 @@
     <row r="69">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bee2280453b94cfc</t>
+          <t xml:space="preserve">c3ab42d597a745d0</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -5001,12 +5001,12 @@
     <row r="70">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bb843da7325e401c</t>
+          <t xml:space="preserve">6add5bf29c0b43a1</t>
         </is>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -5059,12 +5059,12 @@
     <row r="71">
       <c r="A71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eb89032ac49c49c1</t>
+          <t xml:space="preserve">02cc2f2753254651</t>
         </is>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -5117,12 +5117,12 @@
     <row r="72">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bf970f255f3740f5</t>
+          <t xml:space="preserve">20e1affeddb346db</t>
         </is>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -5175,12 +5175,12 @@
     <row r="73">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6559319ffe5f44fc</t>
+          <t xml:space="preserve">d045b82a249f4c13</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -5233,12 +5233,12 @@
     <row r="74">
       <c r="A74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">419f3351d18249de</t>
+          <t xml:space="preserve">752bff991a984810</t>
         </is>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -5291,12 +5291,12 @@
     <row r="75">
       <c r="A75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">963f86e3ad254474</t>
+          <t xml:space="preserve">4a09554cb9cd4a9d</t>
         </is>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -5349,12 +5349,12 @@
     <row r="76">
       <c r="A76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">389b677ffa0d46c8</t>
+          <t xml:space="preserve">801c36cb15ad49c5</t>
         </is>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -5407,12 +5407,12 @@
     <row r="77">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6d92cb51672040f8</t>
+          <t xml:space="preserve">29e07aa8c23e4fbb</t>
         </is>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -5465,12 +5465,12 @@
     <row r="78">
       <c r="A78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cba8f8d3f90f4d21</t>
+          <t xml:space="preserve">a75030ca2a074ba9</t>
         </is>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -5523,12 +5523,12 @@
     <row r="79">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">081eeb6d27fc4a52</t>
+          <t xml:space="preserve">831f261fd38146f3</t>
         </is>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -5581,12 +5581,12 @@
     <row r="80">
       <c r="A80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b3e9a9ce9e004bb2</t>
+          <t xml:space="preserve">38197e6c9a8d4b7a</t>
         </is>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -5639,12 +5639,12 @@
     <row r="81">
       <c r="A81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ae53055f16aa4333</t>
+          <t xml:space="preserve">c2337f9480f9428c</t>
         </is>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -5697,12 +5697,12 @@
     <row r="82">
       <c r="A82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c0c9ceb295e240c0</t>
+          <t xml:space="preserve">d4cbc607f0c14d57</t>
         </is>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -5755,12 +5755,12 @@
     <row r="83">
       <c r="A83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d6a32fb5ed884e78</t>
+          <t xml:space="preserve">106f5b8999e94957</t>
         </is>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -5813,12 +5813,12 @@
     <row r="84">
       <c r="A84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fb1e78a659054806</t>
+          <t xml:space="preserve">1be8da135ffd4c2c</t>
         </is>
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -5871,12 +5871,12 @@
     <row r="85">
       <c r="A85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f133936cc9324cbb</t>
+          <t xml:space="preserve">a027bca7bfa84a8e</t>
         </is>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -5929,12 +5929,12 @@
     <row r="86">
       <c r="A86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1e5f2ca5746747ab</t>
+          <t xml:space="preserve">e60eca24b3844bb9</t>
         </is>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -5987,12 +5987,12 @@
     <row r="87">
       <c r="A87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">12f2c21addcc4287</t>
+          <t xml:space="preserve">b64258bd017c4d6f</t>
         </is>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -6045,12 +6045,12 @@
     <row r="88">
       <c r="A88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">02295b9817fe43ac</t>
+          <t xml:space="preserve">db935670fca74246</t>
         </is>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -6103,12 +6103,12 @@
     <row r="89">
       <c r="A89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">61cd8dc953914e2a</t>
+          <t xml:space="preserve">a4dc4985d2d443db</t>
         </is>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -6161,12 +6161,12 @@
     <row r="90">
       <c r="A90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d3017c8a1e3542cd</t>
+          <t xml:space="preserve">1c2597014f5546c5</t>
         </is>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -6219,12 +6219,12 @@
     <row r="91">
       <c r="A91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">672ed99b172c4955</t>
+          <t xml:space="preserve">f93da2cd41454ea0</t>
         </is>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -6277,12 +6277,12 @@
     <row r="92">
       <c r="A92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3f89ad08e0864e1d</t>
+          <t xml:space="preserve">649c045b52794c29</t>
         </is>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -6335,12 +6335,12 @@
     <row r="93">
       <c r="A93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f661327d1e354a0a</t>
+          <t xml:space="preserve">86d35851308b44ac</t>
         </is>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -6393,12 +6393,12 @@
     <row r="94">
       <c r="A94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ba8fc7598c794284</t>
+          <t xml:space="preserve">f921288456184860</t>
         </is>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -6451,12 +6451,12 @@
     <row r="95">
       <c r="A95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c63aa8a8e7af4636</t>
+          <t xml:space="preserve">45c326ea4857464c</t>
         </is>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e295f92f55be4af5</t>
+          <t xml:space="preserve">7b4d61b1556a4e87</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Add explicit stair support geometric inspection and project evidence (Thai BIM 0.18.0)
</commit_message>
<xml_diff>
--- a/examples/extensions/thai_bim/examples/slab-reinforcement-BBS.xlsx
+++ b/examples/extensions/thai_bim/examples/slab-reinforcement-BBS.xlsx
@@ -164,12 +164,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-4E26E3FCA12B</t>
+          <t xml:space="preserve">B-4068504360E9</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -181,26 +181,26 @@
         <v>12.0</v>
       </c>
       <c r="E2" s="2">
-        <v>11.0</v>
+        <v>7.0</v>
       </c>
       <c r="F2" s="2">
-        <v>0.5</v>
+        <v>2.9380000001999997</v>
       </c>
       <c r="G2" s="2">
-        <v>5.5</v>
+        <v>20.5660000014</v>
       </c>
       <c r="H2" s="2">
         <v>0.8878140839044755</v>
       </c>
       <c r="I2" s="2">
-        <v>4.882977461474615</v>
+        <v>18.258784450822382</v>
       </c>
       <c r="J2" s="2">
         <v>6.0</v>
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">500.000</t>
+          <t xml:space="preserve">2938.000</t>
         </is>
       </c>
       <c r="L2" s="0" t="inlineStr">
@@ -213,7 +213,7 @@
       </c>
       <c r="N2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="O2" s="0" t="inlineStr">
@@ -238,12 +238,12 @@
       </c>
       <c r="S2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">End dowel Start</t>
+          <t xml:space="preserve">Main Bottom</t>
         </is>
       </c>
       <c r="U2" s="0" t="inlineStr">
@@ -255,12 +255,12 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-A359E7AF0105</t>
+          <t xml:space="preserve">B-54ED5FEFBD3F</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -269,29 +269,29 @@
         </is>
       </c>
       <c r="D3" s="2">
-        <v>3.0</v>
+        <v>12.0</v>
       </c>
       <c r="E3" s="2">
-        <v>21.0</v>
+        <v>14.0</v>
       </c>
       <c r="F3" s="2">
-        <v>1.9470000002</v>
+        <v>1.9380000002</v>
       </c>
       <c r="G3" s="2">
-        <v>40.887000004200004</v>
+        <v>27.132000002799998</v>
       </c>
       <c r="H3" s="2">
-        <v>0.05548838024402972</v>
+        <v>0.8878140839044755</v>
       </c>
       <c r="I3" s="2">
-        <v>2.2687534032706944</v>
+        <v>24.08817172698211</v>
       </c>
       <c r="J3" s="2">
-        <v>1.5</v>
+        <v>6.0</v>
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1947.000</t>
+          <t xml:space="preserve">1938.000</t>
         </is>
       </c>
       <c r="L3" s="0" t="inlineStr">
@@ -304,7 +304,7 @@
       </c>
       <c r="N3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="O3" s="0" t="inlineStr">
@@ -329,29 +329,29 @@
       </c>
       <c r="S3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wire mesh B</t>
+          <t xml:space="preserve">Main Bottom</t>
         </is>
       </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-D6B42F9271BC</t>
+          <t xml:space="preserve">B-74C88A2DAA56</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -360,29 +360,29 @@
         </is>
       </c>
       <c r="D4" s="2">
-        <v>12.0</v>
+        <v>6.0</v>
       </c>
       <c r="E4" s="2">
-        <v>11.0</v>
+        <v>1.0</v>
       </c>
       <c r="F4" s="2">
-        <v>0.5</v>
+        <v>0.9456013470417681</v>
       </c>
       <c r="G4" s="2">
-        <v>5.5</v>
+        <v>0.9456013470417681</v>
       </c>
       <c r="H4" s="2">
-        <v>0.8878140839044755</v>
+        <v>0.22195352097611887</v>
       </c>
       <c r="I4" s="2">
-        <v>4.882977461474615</v>
+        <v>0.20987954841568132</v>
       </c>
       <c r="J4" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">500.000</t>
+          <t xml:space="preserve">945.601</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
@@ -395,7 +395,7 @@
       </c>
       <c r="N4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="O4" s="0" t="inlineStr">
@@ -420,12 +420,12 @@
       </c>
       <c r="S4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">End dowel End</t>
+          <t xml:space="preserve">Distribution Bottom</t>
         </is>
       </c>
       <c r="U4" s="0" t="inlineStr">
@@ -437,12 +437,12 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
+          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-DCB1303E84A9</t>
+          <t xml:space="preserve">B-C737C991D2B6</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -451,29 +451,29 @@
         </is>
       </c>
       <c r="D5" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.9440000002</v>
+      </c>
+      <c r="G5" s="2">
+        <v>4.720000001</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0.22195352097611887</v>
+      </c>
+      <c r="I5" s="2">
+        <v>1.0476206192292348</v>
+      </c>
+      <c r="J5" s="2">
         <v>3.0</v>
       </c>
-      <c r="E5" s="2">
-        <v>14.0</v>
-      </c>
-      <c r="F5" s="2">
-        <v>2.9470000002</v>
-      </c>
-      <c r="G5" s="2">
-        <v>41.2580000028</v>
-      </c>
-      <c r="H5" s="2">
-        <v>0.05548838024402972</v>
-      </c>
-      <c r="I5" s="2">
-        <v>2.289339592263546</v>
-      </c>
-      <c r="J5" s="2">
-        <v>1.5</v>
-      </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2947.000</t>
+          <t xml:space="preserve">944.000</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="N5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="O5" s="0" t="inlineStr">
@@ -511,17 +511,17 @@
       </c>
       <c r="S5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precast</t>
+          <t xml:space="preserve">One-way</t>
         </is>
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wire mesh A</t>
+          <t xml:space="preserve">Distribution Bottom</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-4068504360E9</t>
+          <t xml:space="preserve">B-EC740FDBD18C</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -542,29 +542,29 @@
         </is>
       </c>
       <c r="D6" s="2">
-        <v>12.0</v>
+        <v>6.0</v>
       </c>
       <c r="E6" s="2">
-        <v>7.0</v>
+        <v>10.0</v>
       </c>
       <c r="F6" s="2">
-        <v>2.9380000001999997</v>
+        <v>2.9440000002</v>
       </c>
       <c r="G6" s="2">
-        <v>20.5660000014</v>
+        <v>29.440000001999998</v>
       </c>
       <c r="H6" s="2">
-        <v>0.8878140839044755</v>
+        <v>0.22195352097611887</v>
       </c>
       <c r="I6" s="2">
-        <v>18.258784450822382</v>
+        <v>6.534311657980847</v>
       </c>
       <c r="J6" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2938.000</t>
+          <t xml:space="preserve">2944.000</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="N6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="O6" s="0" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="T6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main Bottom</t>
+          <t xml:space="preserve">Distribution Bottom</t>
         </is>
       </c>
       <c r="U6" s="0" t="inlineStr">
@@ -619,12 +619,12 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-54ED5FEFBD3F</t>
+          <t xml:space="preserve">B-4E26E3FCA12B</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -636,26 +636,26 @@
         <v>12.0</v>
       </c>
       <c r="E7" s="2">
-        <v>14.0</v>
+        <v>11.0</v>
       </c>
       <c r="F7" s="2">
-        <v>1.9380000002</v>
+        <v>0.5</v>
       </c>
       <c r="G7" s="2">
-        <v>27.132000002799998</v>
+        <v>5.5</v>
       </c>
       <c r="H7" s="2">
         <v>0.8878140839044755</v>
       </c>
       <c r="I7" s="2">
-        <v>24.08817172698211</v>
+        <v>4.882977461474615</v>
       </c>
       <c r="J7" s="2">
         <v>6.0</v>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1938.000</t>
+          <t xml:space="preserve">500.000</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="N7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="O7" s="0" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="S7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main Bottom</t>
+          <t xml:space="preserve">End dowel Start</t>
         </is>
       </c>
       <c r="U7" s="0" t="inlineStr">
@@ -710,12 +710,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-74C88A2DAA56</t>
+          <t xml:space="preserve">B-A359E7AF0105</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -724,29 +724,29 @@
         </is>
       </c>
       <c r="D8" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="E8" s="2">
-        <v>1.0</v>
+        <v>21.0</v>
       </c>
       <c r="F8" s="2">
-        <v>0.9456013470417681</v>
+        <v>1.9470000002</v>
       </c>
       <c r="G8" s="2">
-        <v>0.9456013470417681</v>
+        <v>40.887000004200004</v>
       </c>
       <c r="H8" s="2">
-        <v>0.22195352097611887</v>
+        <v>0.05548838024402972</v>
       </c>
       <c r="I8" s="2">
-        <v>0.20987954841568132</v>
+        <v>2.2687534032706944</v>
       </c>
       <c r="J8" s="2">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">945.601</t>
+          <t xml:space="preserve">1947.000</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="N8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="O8" s="0" t="inlineStr">
@@ -784,29 +784,29 @@
       </c>
       <c r="S8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution Bottom</t>
+          <t xml:space="preserve">Wire mesh B</t>
         </is>
       </c>
       <c r="U8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-C737C991D2B6</t>
+          <t xml:space="preserve">B-D6B42F9271BC</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -815,29 +815,29 @@
         </is>
       </c>
       <c r="D9" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="E9" s="2">
+        <v>11.0</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G9" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0.8878140839044755</v>
+      </c>
+      <c r="I9" s="2">
+        <v>4.882977461474615</v>
+      </c>
+      <c r="J9" s="2">
         <v>6.0</v>
       </c>
-      <c r="E9" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="F9" s="2">
-        <v>0.9440000002</v>
-      </c>
-      <c r="G9" s="2">
-        <v>4.720000001</v>
-      </c>
-      <c r="H9" s="2">
-        <v>0.22195352097611887</v>
-      </c>
-      <c r="I9" s="2">
-        <v>1.0476206192292348</v>
-      </c>
-      <c r="J9" s="2">
-        <v>3.0</v>
-      </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">944.000</t>
+          <t xml:space="preserve">500.000</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="N9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="O9" s="0" t="inlineStr">
@@ -875,12 +875,12 @@
       </c>
       <c r="S9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution Bottom</t>
+          <t xml:space="preserve">End dowel End</t>
         </is>
       </c>
       <c r="U9" s="0" t="inlineStr">
@@ -892,12 +892,12 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">พื้นทางเดียวรูปเว้า</t>
+          <t xml:space="preserve">พื้นสองทาง / พื้นสำเร็จ</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-EC740FDBD18C</t>
+          <t xml:space="preserve">B-DCB1303E84A9</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -906,29 +906,29 @@
         </is>
       </c>
       <c r="D10" s="2">
-        <v>6.0</v>
+        <v>3.0</v>
       </c>
       <c r="E10" s="2">
-        <v>10.0</v>
+        <v>14.0</v>
       </c>
       <c r="F10" s="2">
-        <v>2.9440000002</v>
+        <v>2.9470000002</v>
       </c>
       <c r="G10" s="2">
-        <v>29.440000001999998</v>
+        <v>41.2580000028</v>
       </c>
       <c r="H10" s="2">
-        <v>0.22195352097611887</v>
+        <v>0.05548838024402972</v>
       </c>
       <c r="I10" s="2">
-        <v>6.534311657980847</v>
+        <v>2.289339592263546</v>
       </c>
       <c r="J10" s="2">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2944.000</t>
+          <t xml:space="preserve">2947.000</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="N10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="O10" s="0" t="inlineStr">
@@ -966,17 +966,17 @@
       </c>
       <c r="S10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-way</t>
+          <t xml:space="preserve">Precast</t>
         </is>
       </c>
       <c r="T10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution Bottom</t>
+          <t xml:space="preserve">Wire mesh A</t>
         </is>
       </c>
       <c r="U10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ไวร์เมชตัวอย่าง 3 mm</t>
         </is>
       </c>
     </row>
@@ -1057,12 +1057,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0d796e43a5dc458c</t>
+          <t xml:space="preserve">fd062e0d84c74b4b</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -1115,12 +1115,12 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d2bf9e94e149462f</t>
+          <t xml:space="preserve">544743f332c946d0</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -1173,12 +1173,12 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2463f9bd593e425f</t>
+          <t xml:space="preserve">95550e7248c6400c</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -1231,12 +1231,12 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">95ae9e30887d416a</t>
+          <t xml:space="preserve">c5cff2d1fb6c4278</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -1289,12 +1289,12 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b7b224d81f3a4258</t>
+          <t xml:space="preserve">ae0f7f1af0fe4534</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -1347,12 +1347,12 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8a15ddd650264220</t>
+          <t xml:space="preserve">9791c2b7cac447cb</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -1405,12 +1405,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">da5bec25e7484abc</t>
+          <t xml:space="preserve">2bef405ab5b6409b</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -1463,12 +1463,12 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">666118299db946b9</t>
+          <t xml:space="preserve">750e5e52a38a4013</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -1521,12 +1521,12 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2fd40d8896a146c4</t>
+          <t xml:space="preserve">0fe5945ef66f4a95</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -1579,12 +1579,12 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e15111740c9f4bfa</t>
+          <t xml:space="preserve">0f4be505e7574972</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -1637,12 +1637,12 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">01c49070802540e3</t>
+          <t xml:space="preserve">94f5424b5e3545a3</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -1695,12 +1695,12 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2e73926c88274f2d</t>
+          <t xml:space="preserve">0df74ae42cb74df3</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -1753,12 +1753,12 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1afa20a805014b9a</t>
+          <t xml:space="preserve">a8905968dcb34d86</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -1811,12 +1811,12 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4ca389f43f9040c2</t>
+          <t xml:space="preserve">75daefcba55e4f6a</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -1869,12 +1869,12 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">80e6dcda1d6d496a</t>
+          <t xml:space="preserve">2d7f7d1fb1dd4236</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -1927,12 +1927,12 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">dcb9d2742559441b</t>
+          <t xml:space="preserve">7f2e9681b02f408e</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1985,12 +1985,12 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f9c59b4086ed490b</t>
+          <t xml:space="preserve">7f32ee80d0c74c2f</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -2043,12 +2043,12 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3d5f6aa53b46474f</t>
+          <t xml:space="preserve">206c38c61cd14d12</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -2101,12 +2101,12 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">375ac762864d433a</t>
+          <t xml:space="preserve">0f36b744aa214697</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -2159,12 +2159,12 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a1573a96c8894b04</t>
+          <t xml:space="preserve">bff20d1a05d54c03</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -2217,12 +2217,12 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d663efbf22464951</t>
+          <t xml:space="preserve">824656252a904a7a</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -2275,12 +2275,12 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">15c1c4e0d1fb43c1</t>
+          <t xml:space="preserve">21e0807dbc144107</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -2333,12 +2333,12 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">342a50776f01483c</t>
+          <t xml:space="preserve">92f8fd7b43c74629</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -2391,12 +2391,12 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">58b7fa1ca7d74f65</t>
+          <t xml:space="preserve">8a510277961342e9</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -2449,12 +2449,12 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fc7e2015960d47ce</t>
+          <t xml:space="preserve">18385031153440f1</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -2507,12 +2507,12 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bac15b3a3f45440b</t>
+          <t xml:space="preserve">b612c3a44f3c4b2f</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -2565,12 +2565,12 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">188d0989beff4d65</t>
+          <t xml:space="preserve">6379aed398a74ec1</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -2623,12 +2623,12 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">112cb946752340a5</t>
+          <t xml:space="preserve">9937fb3433a44476</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -2681,12 +2681,12 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">90ef75e0bbfe4424</t>
+          <t xml:space="preserve">df99e75943b94946</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -2739,12 +2739,12 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">601ddae8e63944e8</t>
+          <t xml:space="preserve">d2748d1b2e2f4512</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -2797,12 +2797,12 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5f735eea602f4ff7</t>
+          <t xml:space="preserve">53fd61b5a2394621</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -2855,12 +2855,12 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e8a5efc1e62f4f5e</t>
+          <t xml:space="preserve">30673ab7b43e4461</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2913,12 +2913,12 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bb6be0baa44343d9</t>
+          <t xml:space="preserve">fcff58c8550a4e86</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2971,12 +2971,12 @@
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c94c8dc519704290</t>
+          <t xml:space="preserve">5f5ea3d813da448c</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -3029,12 +3029,12 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c9ceb61d59e24a0c</t>
+          <t xml:space="preserve">c28cf704f2224644</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -3087,12 +3087,12 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">40a5c132c8454804</t>
+          <t xml:space="preserve">f0ed2696a86f45c1</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -3145,12 +3145,12 @@
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0e72cbc6fc6f4758</t>
+          <t xml:space="preserve">aec5fdfda5f24865</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ac69a8dd966845d7</t>
+          <t xml:space="preserve">85cddc978446403f</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -3203,12 +3203,12 @@
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3ec414a1b88845e7</t>
+          <t xml:space="preserve">59e1ebb4b1f749da</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -3261,12 +3261,12 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aa225fbc2c0644e3</t>
+          <t xml:space="preserve">a6b247c4c07d47b0</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -3319,12 +3319,12 @@
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a5601e68369747b5</t>
+          <t xml:space="preserve">2a88a13437644117</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -3377,12 +3377,12 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">307743a2f46c4f6c</t>
+          <t xml:space="preserve">788c445723cd4153</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bad7b266ed77445f</t>
+          <t xml:space="preserve">e0f06313211546ea</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -3493,12 +3493,12 @@
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2ff59de791ae4b7b</t>
+          <t xml:space="preserve">9bbb284b70ab41fc</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -3551,12 +3551,12 @@
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">db8d8a8c24dd42ec</t>
+          <t xml:space="preserve">ec385df2d22d4f5d</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -3609,12 +3609,12 @@
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5a052fb081c34077</t>
+          <t xml:space="preserve">4b8513939a8e4606</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -3667,12 +3667,12 @@
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">405a417046d24628</t>
+          <t xml:space="preserve">16f5802237ba4b53</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -3725,12 +3725,12 @@
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1870a730ffa54191</t>
+          <t xml:space="preserve">8486bd0bc90f4589</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -3783,12 +3783,12 @@
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e6e90c1461d74666</t>
+          <t xml:space="preserve">70251d307e394d27</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -3841,12 +3841,12 @@
     <row r="50">
       <c r="A50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">416df7a6e20848ab</t>
+          <t xml:space="preserve">ca6b99e32f3745be</t>
         </is>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3899,12 +3899,12 @@
     <row r="51">
       <c r="A51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f0687d49f0674176</t>
+          <t xml:space="preserve">618c6a1b4bfc4565</t>
         </is>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3957,12 +3957,12 @@
     <row r="52">
       <c r="A52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f62c5ed57d2e4dee</t>
+          <t xml:space="preserve">d726cb9ad4fd4898</t>
         </is>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -4015,12 +4015,12 @@
     <row r="53">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4092b0cf9d3f4564</t>
+          <t xml:space="preserve">60d4f0d39587404c</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -4073,12 +4073,12 @@
     <row r="54">
       <c r="A54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a4efe3896afe4fef</t>
+          <t xml:space="preserve">be647c6739814eee</t>
         </is>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -4131,12 +4131,12 @@
     <row r="55">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">41ac9eb7e5cc4e5a</t>
+          <t xml:space="preserve">2ca096ba67e64ccb</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -4189,12 +4189,12 @@
     <row r="56">
       <c r="A56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">76bbb129bfe4415c</t>
+          <t xml:space="preserve">6dd47d21dbb1443c</t>
         </is>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -4247,12 +4247,12 @@
     <row r="57">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">88801c1f42e646e1</t>
+          <t xml:space="preserve">6ed558d3aa134e0c</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -4305,12 +4305,12 @@
     <row r="58">
       <c r="A58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5be36060bb6f483b</t>
+          <t xml:space="preserve">b296434f6bd64441</t>
         </is>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -4363,12 +4363,12 @@
     <row r="59">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aac1760efebf4d1c</t>
+          <t xml:space="preserve">7f04baf1f3104930</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -4421,12 +4421,12 @@
     <row r="60">
       <c r="A60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e69b1fcc4ee34039</t>
+          <t xml:space="preserve">57e96a85656c4b2c</t>
         </is>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -4479,12 +4479,12 @@
     <row r="61">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">90de4dc1c46b449d</t>
+          <t xml:space="preserve">dcdc3f73d8894f67</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -4537,12 +4537,12 @@
     <row r="62">
       <c r="A62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">603832b5897b488d</t>
+          <t xml:space="preserve">ef755cf2e6a6475b</t>
         </is>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -4595,12 +4595,12 @@
     <row r="63">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1900ba1079c34ecf</t>
+          <t xml:space="preserve">cb1005b7d3904764</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -4653,12 +4653,12 @@
     <row r="64">
       <c r="A64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a68e9c0dc0bd46c2</t>
+          <t xml:space="preserve">d75079a8cefa4dc4</t>
         </is>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -4711,12 +4711,12 @@
     <row r="65">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e40399b122a94226</t>
+          <t xml:space="preserve">13e3c0f4e54940d7</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -4769,12 +4769,12 @@
     <row r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">89efea1cf8b24b09</t>
+          <t xml:space="preserve">07e1233654744237</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -4827,12 +4827,12 @@
     <row r="67">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d305baf593384870</t>
+          <t xml:space="preserve">a6eafac366e34273</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4885,12 +4885,12 @@
     <row r="68">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">fe712f03b99843a1</t>
+          <t xml:space="preserve">c61e552802f94172</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -4943,12 +4943,12 @@
     <row r="69">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c3ab42d597a745d0</t>
+          <t xml:space="preserve">df127df697bd40a9</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -5001,12 +5001,12 @@
     <row r="70">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6add5bf29c0b43a1</t>
+          <t xml:space="preserve">4419a902a79a4fe9</t>
         </is>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -5059,12 +5059,12 @@
     <row r="71">
       <c r="A71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">02cc2f2753254651</t>
+          <t xml:space="preserve">9c92ac9a229045fc</t>
         </is>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -5117,12 +5117,12 @@
     <row r="72">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">20e1affeddb346db</t>
+          <t xml:space="preserve">35f1d38f27b24cba</t>
         </is>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -5175,12 +5175,12 @@
     <row r="73">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d045b82a249f4c13</t>
+          <t xml:space="preserve">dcefe1f914af4892</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -5233,12 +5233,12 @@
     <row r="74">
       <c r="A74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">752bff991a984810</t>
+          <t xml:space="preserve">47f87ec0bc3e41fc</t>
         </is>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -5291,12 +5291,12 @@
     <row r="75">
       <c r="A75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4a09554cb9cd4a9d</t>
+          <t xml:space="preserve">67c2f4cb7fb04d60</t>
         </is>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -5349,12 +5349,12 @@
     <row r="76">
       <c r="A76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">801c36cb15ad49c5</t>
+          <t xml:space="preserve">32529d5bab354894</t>
         </is>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -5407,12 +5407,12 @@
     <row r="77">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">29e07aa8c23e4fbb</t>
+          <t xml:space="preserve">733baa3368c54dff</t>
         </is>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -5465,12 +5465,12 @@
     <row r="78">
       <c r="A78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a75030ca2a074ba9</t>
+          <t xml:space="preserve">0d03f4333fb84888</t>
         </is>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -5523,12 +5523,12 @@
     <row r="79">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">831f261fd38146f3</t>
+          <t xml:space="preserve">ddda4232d53d4008</t>
         </is>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -5581,12 +5581,12 @@
     <row r="80">
       <c r="A80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">38197e6c9a8d4b7a</t>
+          <t xml:space="preserve">2d89b6fdbba741cc</t>
         </is>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -5639,12 +5639,12 @@
     <row r="81">
       <c r="A81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c2337f9480f9428c</t>
+          <t xml:space="preserve">a7bbc1249ae2482f</t>
         </is>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -5697,12 +5697,12 @@
     <row r="82">
       <c r="A82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d4cbc607f0c14d57</t>
+          <t xml:space="preserve">aa20c9312a944d73</t>
         </is>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -5755,12 +5755,12 @@
     <row r="83">
       <c r="A83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">106f5b8999e94957</t>
+          <t xml:space="preserve">5666d7491c0c4982</t>
         </is>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -5813,12 +5813,12 @@
     <row r="84">
       <c r="A84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1be8da135ffd4c2c</t>
+          <t xml:space="preserve">5c1d9d650b3b455d</t>
         </is>
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -5871,12 +5871,12 @@
     <row r="85">
       <c r="A85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a027bca7bfa84a8e</t>
+          <t xml:space="preserve">89cd526a51704ad6</t>
         </is>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -5929,12 +5929,12 @@
     <row r="86">
       <c r="A86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e60eca24b3844bb9</t>
+          <t xml:space="preserve">7cb8ad814c844d53</t>
         </is>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -5987,12 +5987,12 @@
     <row r="87">
       <c r="A87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b64258bd017c4d6f</t>
+          <t xml:space="preserve">0d4c6d678d214edb</t>
         </is>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -6045,12 +6045,12 @@
     <row r="88">
       <c r="A88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">db935670fca74246</t>
+          <t xml:space="preserve">d376f87901564a2c</t>
         </is>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -6103,12 +6103,12 @@
     <row r="89">
       <c r="A89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a4dc4985d2d443db</t>
+          <t xml:space="preserve">efbc209d2aab4f60</t>
         </is>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -6161,12 +6161,12 @@
     <row r="90">
       <c r="A90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1c2597014f5546c5</t>
+          <t xml:space="preserve">b021832a411c4507</t>
         </is>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -6219,12 +6219,12 @@
     <row r="91">
       <c r="A91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f93da2cd41454ea0</t>
+          <t xml:space="preserve">0e3edb6d46324af8</t>
         </is>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -6277,12 +6277,12 @@
     <row r="92">
       <c r="A92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">649c045b52794c29</t>
+          <t xml:space="preserve">3c85068b21e2448c</t>
         </is>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -6335,12 +6335,12 @@
     <row r="93">
       <c r="A93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">86d35851308b44ac</t>
+          <t xml:space="preserve">d37ca7fa94014bc4</t>
         </is>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -6393,12 +6393,12 @@
     <row r="94">
       <c r="A94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f921288456184860</t>
+          <t xml:space="preserve">0d3b739d9e32450d</t>
         </is>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -6451,12 +6451,12 @@
     <row r="95">
       <c r="A95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">45c326ea4857464c</t>
+          <t xml:space="preserve">e8c7ca5024fe45e0</t>
         </is>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7b4d61b1556a4e87</t>
+          <t xml:space="preserve">ea6b17a682804e96</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">

</xml_diff>